<commit_message>
added company layer to items master data
</commit_message>
<xml_diff>
--- a/template/Item_Template.xlsx
+++ b/template/Item_Template.xlsx
@@ -27,10 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
-  <si>
-    <t>Company</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>Item Code</t>
   </si>
@@ -1014,15 +1011,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:F1"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15" outlineLevelCol="5"/>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15" outlineLevelCol="4"/>
   <cols>
-    <col min="2" max="2" width="12.8740740740741" customWidth="1"/>
-    <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="16.5555555555556" customWidth="1"/>
+    <col min="1" max="1" width="12.8740740740741" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="16.5555555555556" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.75" spans="1:6">
+    <row r="1" ht="15.75" spans="1:5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1038,9 +1035,6 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>